<commit_message>
update farmland npp case
</commit_message>
<xml_diff>
--- a/gcmc_data_codes/Case of net primary productivity study/Case of net primary productivity study.xlsx
+++ b/gcmc_data_codes/Case of net primary productivity study/Case of net primary productivity study.xlsx
@@ -392,10 +392,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.239742883379247</v>
+        <v>0.599585262345679</v>
       </c>
       <c r="D2">
-        <v>1.57180651321647E-17</v>
+        <v>0.009477523412991826</v>
       </c>
     </row>
     <row r="3">
@@ -410,10 +410,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.2060238751147842</v>
+        <v>0.5575810185185185</v>
       </c>
       <c r="D3">
-        <v>6.525043626699835E-25</v>
+        <v>0.1389266748189295</v>
       </c>
     </row>
     <row r="4">
@@ -428,10 +428,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.4287970615243343</v>
+        <v>0.7325424382716049</v>
       </c>
       <c r="D4">
-        <v>0.0470687916497408</v>
+        <v>2.978542382881651E-11</v>
       </c>
     </row>
     <row r="5">
@@ -446,10 +446,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.4322130394857668</v>
+        <v>0.7235725308641975</v>
       </c>
       <c r="D5">
-        <v>0.05956945786229592</v>
+        <v>2.734369813090459E-10</v>
       </c>
     </row>
     <row r="6">
@@ -464,10 +464,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.3222038567493113</v>
+        <v>0.6616994598765432</v>
       </c>
       <c r="D6">
-        <v>1.261609306669625E-07</v>
+        <v>1.485632059595207E-05</v>
       </c>
     </row>
     <row r="7">
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.2725068870523416</v>
+        <v>0.6358989197530864</v>
       </c>
       <c r="D7">
-        <v>5.041517325850549E-13</v>
+        <v>0.0003248357205360693</v>
       </c>
     </row>
   </sheetData>
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.8324397811656905</v>
+        <v>0.6816744771994</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.7989642933404404</v>
+        <v>0.6834700653500174</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.7143327286488832</v>
+        <v>0.6223444863156565</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.6559515226195394</v>
+        <v>0.5224668885827265</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.7672520290787253</v>
+        <v>0.6322412475686654</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.8053771235694317</v>
+        <v>0.6510014176420699</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -672,10 +672,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.7906236204443422</v>
+        <v>0.8018719322811553</v>
       </c>
       <c r="D2">
-        <v>9.574992216403358E-321</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -690,10 +690,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.6767460761540719</v>
+        <v>0.6679425886483285</v>
       </c>
       <c r="D3">
-        <v>2.459234976177667E-201</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -708,10 +708,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.7906236204443422</v>
+        <v>0.8018719322811553</v>
       </c>
       <c r="D4">
-        <v>3.191664072134453E-321</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -726,10 +726,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.7834559178342438</v>
+        <v>0.7761627037245852</v>
       </c>
       <c r="D5">
-        <v>2.801567142578441E-311</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -744,10 +744,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.6767460761540719</v>
+        <v>0.6679425886483285</v>
       </c>
       <c r="D6">
-        <v>2.459234976177667E-201</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -762,10 +762,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.7834559178342438</v>
+        <v>0.7761627037245852</v>
       </c>
       <c r="D7">
-        <v>1.40078357128922E-311</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -812,10 +812,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.3756260251040425</v>
+        <v>0.3817923884995237</v>
       </c>
       <c r="D2">
-        <v>3.642653099578032E-126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -833,7 +833,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>6.553671515938445E-28</v>
+        <v>1.92638334690847E-169</v>
       </c>
     </row>
     <row r="4">
@@ -851,7 +851,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>3.642653099578032E-126</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -869,7 +869,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>2.31191231028444E-93</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -884,10 +884,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.003965936370808507</v>
+        <v>0.003323124278150534</v>
       </c>
       <c r="D6">
-        <v>6.553671515938445E-28</v>
+        <v>1.92638334690847E-169</v>
       </c>
     </row>
     <row r="7">
@@ -902,10 +902,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.008164496560567478</v>
+        <v>0.008354302550777449</v>
       </c>
       <c r="D7">
-        <v>2.31191231028444E-93</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -952,10 +952,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.6654054331056385</v>
+        <v>0.6844018387403827</v>
       </c>
       <c r="D2">
-        <v>7.72506417666928E-10</v>
+        <v>4.452767785024202E-10</v>
       </c>
     </row>
     <row r="3">
@@ -970,10 +970,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.7054040861800186</v>
+        <v>0.7144418626825814</v>
       </c>
       <c r="D3">
-        <v>5.137835857173083E-10</v>
+        <v>2.014629365567309E-10</v>
       </c>
     </row>
     <row r="4">
@@ -988,10 +988,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.5023683677647043</v>
+        <v>0.4987582320692993</v>
       </c>
       <c r="D4">
-        <v>5.916373439340122E-10</v>
+        <v>1.832813454499295E-10</v>
       </c>
     </row>
     <row r="5">
@@ -1006,10 +1006,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.516754333574873</v>
+        <v>0.5203768220567544</v>
       </c>
       <c r="D5">
-        <v>3.665787554150285E-10</v>
+        <v>8.647696774703555E-10</v>
       </c>
     </row>
     <row r="6">
@@ -1024,10 +1024,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.6720817957056606</v>
+        <v>0.6688227574539</v>
       </c>
       <c r="D6">
-        <v>5.796740930688084E-10</v>
+        <v>8.258056917865957E-10</v>
       </c>
     </row>
     <row r="7">
@@ -1042,10 +1042,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.6923947457456827</v>
+        <v>0.6927814975854476</v>
       </c>
       <c r="D7">
-        <v>6.810004908618973E-10</v>
+        <v>1.843406556415773E-10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>